<commit_message>
Ítems paso a paso para todo el equipo y efectos al golpear con tirada
- comun/asistente-item.js reemplaza al asistente de armas: paso 1 con
  categoría, nombre y descripción en palabras; después solo lo práctico
  según la categoría (armas, defensa y resistencias a crítico, bonos,
  estado al equipar, precio/lugar). Lo usan la ficha, GM Tools (Ítem
  custom y arma del creep), el generador de tiendas y el editor de
  catálogo; los consumibles siguen con su formulario.
- comun/efectos-golpe.js: las armas llevan efectosGolpe (probabilidad en
  1dN y tirada extra opcional). Al tirar el Daño (ficha y creeps) salen
  resaltados en la Mesa y, si tienen porcentaje, se tiran en un pop-up
  (50% = moneda, 25% = d4...). Aplicarlos al rival sigue siendo manual.
- 38 armas del catálogo pasan sus efectos escritos a efectosGolpe; el
  importador y el Excel (columna "Efectos al golpear") los conservan.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -17,7 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Consumibles'!$A$1:$W$147</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$X$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Armas'!$A$1:$Y$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Escudos'!$A$1:$V$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Defensivos'!$A$1:$AI$250</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Accesorios'!$A$1:$V$73</definedName>
@@ -678,11 +678,7 @@
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1911,11 +1907,7 @@
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
       <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1982,11 +1974,7 @@
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
       <c r="V18" t="inlineStr"/>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2053,11 +2041,7 @@
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
       <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2124,11 +2108,7 @@
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
       <c r="V20" t="inlineStr"/>
-      <c r="W20" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2195,11 +2175,7 @@
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
       <c r="V21" t="inlineStr"/>
-      <c r="W21" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2266,11 +2242,7 @@
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2582,11 +2554,7 @@
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr"/>
       <c r="V26" t="inlineStr"/>
-      <c r="W26" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2657,11 +2625,7 @@
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
       <c r="V27" t="inlineStr"/>
-      <c r="W27" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4711,11 +4675,7 @@
       <c r="T53" t="inlineStr"/>
       <c r="U53" t="inlineStr"/>
       <c r="V53" t="inlineStr"/>
-      <c r="W53" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5418,11 +5378,7 @@
       <c r="T62" t="inlineStr"/>
       <c r="U62" t="inlineStr"/>
       <c r="V62" t="inlineStr"/>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5493,11 +5449,7 @@
       <c r="T63" t="inlineStr"/>
       <c r="U63" t="inlineStr"/>
       <c r="V63" t="inlineStr"/>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5568,11 +5520,7 @@
       <c r="T64" t="inlineStr"/>
       <c r="U64" t="inlineStr"/>
       <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5643,11 +5591,7 @@
       <c r="T65" t="inlineStr"/>
       <c r="U65" t="inlineStr"/>
       <c r="V65" t="inlineStr"/>
-      <c r="W65" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5789,11 +5733,7 @@
       <c r="T67" t="inlineStr"/>
       <c r="U67" t="inlineStr"/>
       <c r="V67" t="inlineStr"/>
-      <c r="W67" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5868,11 +5808,7 @@
       <c r="T68" t="inlineStr"/>
       <c r="U68" t="inlineStr"/>
       <c r="V68" t="inlineStr"/>
-      <c r="W68" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5943,11 +5879,7 @@
       <c r="T69" t="inlineStr"/>
       <c r="U69" t="inlineStr"/>
       <c r="V69" t="inlineStr"/>
-      <c r="W69" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7464,11 +7396,7 @@
       <c r="T88" t="inlineStr"/>
       <c r="U88" t="inlineStr"/>
       <c r="V88" t="inlineStr"/>
-      <c r="W88" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7768,11 +7696,7 @@
       <c r="T92" t="inlineStr"/>
       <c r="U92" t="inlineStr"/>
       <c r="V92" t="inlineStr"/>
-      <c r="W92" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7843,11 +7767,7 @@
       <c r="T93" t="inlineStr"/>
       <c r="U93" t="inlineStr"/>
       <c r="V93" t="inlineStr"/>
-      <c r="W93" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10727,11 +10647,7 @@
       <c r="T129" t="inlineStr"/>
       <c r="U129" t="inlineStr"/>
       <c r="V129" t="inlineStr"/>
-      <c r="W129" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -10802,11 +10718,7 @@
       <c r="T130" t="inlineStr"/>
       <c r="U130" t="inlineStr"/>
       <c r="V130" t="inlineStr"/>
-      <c r="W130" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -11809,11 +11721,7 @@
       <c r="T143" t="inlineStr"/>
       <c r="U143" t="inlineStr"/>
       <c r="V143" t="inlineStr"/>
-      <c r="W143" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -12133,11 +12041,7 @@
       </c>
       <c r="U147" t="inlineStr"/>
       <c r="V147" t="inlineStr"/>
-      <c r="W147" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="W147" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:W147"/>
@@ -12151,7 +12055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X90"/>
+  <dimension ref="A1:Y90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12176,8 +12080,9 @@
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="13" customWidth="1" min="21" max="21"/>
     <col width="13" customWidth="1" min="22" max="22"/>
-    <col width="30" customWidth="1" min="23" max="23"/>
-    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -12248,55 +12153,60 @@
       </c>
       <c r="N1" s="2" t="inlineStr">
         <is>
+          <t>Efectos al golpear</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
           <t>PdG</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Crítico %</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>Iniciativa</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
         <is>
           <t>Parry</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="S1" s="2" t="inlineStr">
         <is>
           <t>Fuerza</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>Bloqueo</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
         <is>
           <t>Estado al equipar</t>
         </is>
       </c>
-      <c r="U1" s="2" t="inlineStr">
+      <c r="V1" s="2" t="inlineStr">
         <is>
           <t>HP por turno equipado</t>
         </is>
       </c>
-      <c r="V1" s="2" t="inlineStr">
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>Detalle del estado equipado</t>
         </is>
       </c>
-      <c r="W1" s="2" t="inlineStr">
+      <c r="X1" s="2" t="inlineStr">
         <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
@@ -12357,20 +12267,21 @@
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
-      <c r="S2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="n">
-        <v>0</v>
-      </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr"/>
+      <c r="X2" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -12425,18 +12336,19 @@
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="n">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="n">
         <v>2</v>
       </c>
-      <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
-      <c r="U3" t="n">
-        <v>0</v>
-      </c>
-      <c r="V3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
       <c r="W3" t="inlineStr"/>
       <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -12488,21 +12400,22 @@
         <v>0</v>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="inlineStr"/>
-      <c r="U4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
       <c r="W4" t="inlineStr"/>
       <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -12554,19 +12467,24 @@
         <v>0</v>
       </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
-      <c r="U5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
       <c r="W5" t="inlineStr"/>
       <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -12618,25 +12536,22 @@
         <v>0</v>
       </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="n">
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="n">
         <v>2</v>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
-      <c r="U6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V6" t="inlineStr"/>
+      <c r="U6" t="inlineStr"/>
+      <c r="V6" t="n">
+        <v>0</v>
+      </c>
       <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -12689,20 +12604,21 @@
       </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="n">
-        <v>1</v>
-      </c>
-      <c r="P7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="inlineStr"/>
+      <c r="U7" t="inlineStr"/>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -12756,23 +12672,20 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
-      <c r="P8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="inlineStr"/>
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
       <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -12824,19 +12737,24 @@
         <v>0</v>
       </c>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
-      <c r="U9" t="n">
-        <v>0</v>
-      </c>
-      <c r="V9" t="inlineStr"/>
+      <c r="U9" t="inlineStr"/>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
       <c r="W9" t="inlineStr"/>
       <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12888,19 +12806,24 @@
         <v>0</v>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
-      <c r="U10" t="n">
-        <v>0</v>
-      </c>
-      <c r="V10" t="inlineStr"/>
+      <c r="U10" t="inlineStr"/>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -12952,25 +12875,26 @@
         <v>0</v>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="n">
-        <v>1</v>
-      </c>
-      <c r="T11" t="inlineStr"/>
-      <c r="U11" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" t="inlineStr"/>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
       <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -13022,19 +12946,24 @@
         <v>0</v>
       </c>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
-      <c r="U12" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -13089,12 +13018,13 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
-      <c r="U13" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" t="inlineStr"/>
+      <c r="U13" t="inlineStr"/>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
+      <c r="Y13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -13146,19 +13076,24 @@
         <v>0</v>
       </c>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Sangrado 1/2: Aplicale Sangrado al objetivo.</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
-      <c r="U14" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" t="inlineStr"/>
+      <c r="U14" t="inlineStr"/>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
+      <c r="Y14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -13213,16 +13148,13 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
-      <c r="U15" t="n">
-        <v>0</v>
-      </c>
-      <c r="V15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
       <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X15" t="inlineStr"/>
+      <c r="Y15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -13279,16 +13211,17 @@
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
-      <c r="S16" t="n">
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="n">
         <v>2</v>
       </c>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" t="inlineStr"/>
+      <c r="U16" t="inlineStr"/>
+      <c r="V16" t="n">
+        <v>0</v>
+      </c>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
+      <c r="Y16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -13345,16 +13278,17 @@
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
-      <c r="S17" t="n">
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="n">
         <v>3</v>
       </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="n">
-        <v>0</v>
-      </c>
-      <c r="V17" t="inlineStr"/>
+      <c r="U17" t="inlineStr"/>
+      <c r="V17" t="n">
+        <v>0</v>
+      </c>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
+      <c r="Y17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -13409,12 +13343,13 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
-      <c r="U18" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" t="inlineStr"/>
+      <c r="U18" t="inlineStr"/>
+      <c r="V18" t="n">
+        <v>0</v>
+      </c>
       <c r="W18" t="inlineStr"/>
       <c r="X18" t="inlineStr"/>
+      <c r="Y18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -13466,23 +13401,28 @@
         <v>0</v>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Rompe armadura 1/2: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
-      <c r="U19" t="n">
-        <v>0</v>
-      </c>
-      <c r="V19" t="inlineStr"/>
-      <c r="W19" t="inlineStr">
+      <c r="U19" t="inlineStr"/>
+      <c r="V19" t="n">
+        <v>0</v>
+      </c>
+      <c r="W19" t="inlineStr"/>
+      <c r="X19" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X19" t="inlineStr"/>
+      <c r="Y19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -13534,23 +13474,24 @@
         <v>0</v>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="n">
-        <v>1</v>
-      </c>
-      <c r="O20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
+      <c r="O20" t="n">
+        <v>1</v>
+      </c>
       <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="n">
+        <v>1</v>
+      </c>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
-      <c r="U20" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" t="inlineStr"/>
+      <c r="U20" t="inlineStr"/>
+      <c r="V20" t="n">
+        <v>0</v>
+      </c>
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr"/>
+      <c r="Y20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -13602,21 +13543,22 @@
         <v>0</v>
       </c>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="n">
-        <v>1</v>
-      </c>
-      <c r="O21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
-      <c r="U21" t="n">
-        <v>0</v>
-      </c>
-      <c r="V21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
+      <c r="V21" t="n">
+        <v>0</v>
+      </c>
       <c r="W21" t="inlineStr"/>
       <c r="X21" t="inlineStr"/>
+      <c r="Y21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -13675,16 +13617,17 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="inlineStr"/>
-      <c r="U22" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" t="inlineStr"/>
-      <c r="W22" t="inlineStr">
+      <c r="U22" t="inlineStr"/>
+      <c r="V22" t="n">
+        <v>0</v>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -13739,12 +13682,13 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
-      <c r="U23" t="n">
-        <v>0</v>
-      </c>
-      <c r="V23" t="inlineStr"/>
+      <c r="U23" t="inlineStr"/>
+      <c r="V23" t="n">
+        <v>0</v>
+      </c>
       <c r="W23" t="inlineStr"/>
       <c r="X23" t="inlineStr"/>
+      <c r="Y23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13793,20 +13737,21 @@
       </c>
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr"/>
-      <c r="O24" t="n">
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
         <v>10</v>
       </c>
-      <c r="P24" t="inlineStr"/>
       <c r="Q24" t="inlineStr"/>
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
-      <c r="U24" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="n">
+        <v>0</v>
+      </c>
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13861,18 +13806,19 @@
       <c r="N25" t="inlineStr"/>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="n">
-        <v>1</v>
-      </c>
-      <c r="R25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="n">
+        <v>1</v>
+      </c>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="inlineStr"/>
-      <c r="U25" t="n">
-        <v>0</v>
-      </c>
-      <c r="V25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="n">
+        <v>0</v>
+      </c>
       <c r="W25" t="inlineStr"/>
       <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13927,12 +13873,13 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="inlineStr"/>
-      <c r="U26" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>0</v>
+      </c>
       <c r="W26" t="inlineStr"/>
       <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -13987,12 +13934,13 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="inlineStr"/>
-      <c r="U27" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>0</v>
+      </c>
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14047,16 +13995,13 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="inlineStr"/>
-      <c r="U28" t="n">
-        <v>0</v>
-      </c>
-      <c r="V28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="n">
+        <v>0</v>
+      </c>
       <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14111,16 +14056,13 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="inlineStr"/>
-      <c r="U29" t="n">
-        <v>0</v>
-      </c>
-      <c r="V29" t="inlineStr"/>
+      <c r="U29" t="inlineStr"/>
+      <c r="V29" t="n">
+        <v>0</v>
+      </c>
       <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X29" t="inlineStr"/>
+      <c r="Y29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -14175,12 +14117,13 @@
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="inlineStr"/>
-      <c r="U30" t="n">
-        <v>0</v>
-      </c>
-      <c r="V30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="n">
+        <v>0</v>
+      </c>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -14232,19 +14175,24 @@
         <v>0</v>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Envenenar 1/2: Aplicale Veneno al objetivo.</t>
+        </is>
+      </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="inlineStr"/>
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="inlineStr"/>
-      <c r="U31" t="n">
-        <v>0</v>
-      </c>
-      <c r="V31" t="inlineStr"/>
+      <c r="U31" t="inlineStr"/>
+      <c r="V31" t="n">
+        <v>0</v>
+      </c>
       <c r="W31" t="inlineStr"/>
       <c r="X31" t="inlineStr"/>
+      <c r="Y31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -14297,20 +14245,21 @@
       </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
-      <c r="O32" t="n">
-        <v>1</v>
-      </c>
-      <c r="P32" t="inlineStr"/>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
       <c r="Q32" t="inlineStr"/>
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="inlineStr"/>
-      <c r="U32" t="n">
-        <v>0</v>
-      </c>
-      <c r="V32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="n">
+        <v>0</v>
+      </c>
       <c r="W32" t="inlineStr"/>
       <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -14365,16 +14314,13 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="inlineStr"/>
-      <c r="U33" t="n">
-        <v>0</v>
-      </c>
-      <c r="V33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="n">
+        <v>0</v>
+      </c>
       <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -14426,23 +14372,24 @@
         <v>0</v>
       </c>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr"/>
       <c r="Q34" t="inlineStr"/>
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="inlineStr"/>
-      <c r="U34" t="n">
-        <v>0</v>
-      </c>
-      <c r="V34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="n">
+        <v>0</v>
+      </c>
       <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -14494,19 +14441,24 @@
         <v>0</v>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="inlineStr"/>
-      <c r="U35" t="n">
-        <v>0</v>
-      </c>
-      <c r="V35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="n">
+        <v>0</v>
+      </c>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -14561,12 +14513,13 @@
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="inlineStr"/>
-      <c r="U36" t="n">
-        <v>0</v>
-      </c>
-      <c r="V36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="n">
+        <v>0</v>
+      </c>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
+      <c r="Y36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -14618,19 +14571,24 @@
         <v>0</v>
       </c>
       <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Envenenar 1/2: Aplicale Veneno al objetivo.</t>
+        </is>
+      </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="inlineStr"/>
-      <c r="U37" t="n">
-        <v>0</v>
-      </c>
-      <c r="V37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="n">
+        <v>0</v>
+      </c>
       <c r="W37" t="inlineStr"/>
       <c r="X37" t="inlineStr"/>
+      <c r="Y37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14685,12 +14643,13 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="inlineStr"/>
-      <c r="U38" t="n">
-        <v>0</v>
-      </c>
-      <c r="V38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="n">
+        <v>0</v>
+      </c>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="inlineStr"/>
+      <c r="Y38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -14749,16 +14708,17 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="inlineStr"/>
-      <c r="U39" t="n">
-        <v>0</v>
-      </c>
-      <c r="V39" t="inlineStr"/>
-      <c r="W39" t="inlineStr">
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="n">
+        <v>0</v>
+      </c>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X39" t="inlineStr"/>
+      <c r="Y39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -14810,19 +14770,24 @@
         <v>0</v>
       </c>
       <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Sangrado 1/2: Aplicale Sangrado al objetivo.</t>
+        </is>
+      </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr"/>
       <c r="Q40" t="inlineStr"/>
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="inlineStr"/>
-      <c r="U40" t="n">
-        <v>0</v>
-      </c>
-      <c r="V40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="n">
+        <v>0</v>
+      </c>
       <c r="W40" t="inlineStr"/>
       <c r="X40" t="inlineStr"/>
+      <c r="Y40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -14881,16 +14846,17 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="inlineStr"/>
-      <c r="U41" t="n">
-        <v>0</v>
-      </c>
-      <c r="V41" t="inlineStr"/>
-      <c r="W41" t="inlineStr">
+      <c r="U41" t="inlineStr"/>
+      <c r="V41" t="n">
+        <v>0</v>
+      </c>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X41" t="inlineStr"/>
+      <c r="Y41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -14942,19 +14908,24 @@
         <v>0</v>
       </c>
       <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Rompe armadura 1/2: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr"/>
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="inlineStr"/>
-      <c r="U42" t="n">
-        <v>0</v>
-      </c>
-      <c r="V42" t="inlineStr"/>
+      <c r="U42" t="inlineStr"/>
+      <c r="V42" t="n">
+        <v>0</v>
+      </c>
       <c r="W42" t="inlineStr"/>
       <c r="X42" t="inlineStr"/>
+      <c r="Y42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -15011,16 +14982,17 @@
       <c r="P43" t="inlineStr"/>
       <c r="Q43" t="inlineStr"/>
       <c r="R43" t="inlineStr"/>
-      <c r="S43" t="n">
-        <v>1</v>
-      </c>
-      <c r="T43" t="inlineStr"/>
-      <c r="U43" t="n">
-        <v>0</v>
-      </c>
-      <c r="V43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+      <c r="T43" t="n">
+        <v>1</v>
+      </c>
+      <c r="U43" t="inlineStr"/>
+      <c r="V43" t="n">
+        <v>0</v>
+      </c>
       <c r="W43" t="inlineStr"/>
       <c r="X43" t="inlineStr"/>
+      <c r="Y43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -15079,16 +15051,17 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="inlineStr"/>
-      <c r="U44" t="n">
-        <v>0</v>
-      </c>
-      <c r="V44" t="inlineStr"/>
-      <c r="W44" t="inlineStr">
+      <c r="U44" t="inlineStr"/>
+      <c r="V44" t="n">
+        <v>0</v>
+      </c>
+      <c r="W44" t="inlineStr"/>
+      <c r="X44" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -15147,12 +15120,13 @@
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="inlineStr"/>
-      <c r="U45" t="n">
-        <v>0</v>
-      </c>
-      <c r="V45" t="inlineStr"/>
+      <c r="U45" t="inlineStr"/>
+      <c r="V45" t="n">
+        <v>0</v>
+      </c>
       <c r="W45" t="inlineStr"/>
       <c r="X45" t="inlineStr"/>
+      <c r="Y45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -15209,16 +15183,17 @@
       <c r="P46" t="inlineStr"/>
       <c r="Q46" t="inlineStr"/>
       <c r="R46" t="inlineStr"/>
-      <c r="S46" t="n">
-        <v>1</v>
-      </c>
-      <c r="T46" t="inlineStr"/>
-      <c r="U46" t="n">
-        <v>0</v>
-      </c>
-      <c r="V46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+      <c r="T46" t="n">
+        <v>1</v>
+      </c>
+      <c r="U46" t="inlineStr"/>
+      <c r="V46" t="n">
+        <v>0</v>
+      </c>
       <c r="W46" t="inlineStr"/>
       <c r="X46" t="inlineStr"/>
+      <c r="Y46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -15273,12 +15248,13 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="inlineStr"/>
-      <c r="U47" t="n">
-        <v>0</v>
-      </c>
-      <c r="V47" t="inlineStr"/>
+      <c r="U47" t="inlineStr"/>
+      <c r="V47" t="n">
+        <v>0</v>
+      </c>
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr"/>
+      <c r="Y47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -15332,19 +15308,20 @@
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr"/>
       <c r="O48" t="inlineStr"/>
-      <c r="P48" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="n">
+        <v>1</v>
+      </c>
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="inlineStr"/>
-      <c r="U48" t="n">
-        <v>0</v>
-      </c>
-      <c r="V48" t="inlineStr"/>
+      <c r="U48" t="inlineStr"/>
+      <c r="V48" t="n">
+        <v>0</v>
+      </c>
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr"/>
+      <c r="Y48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -15403,16 +15380,17 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="inlineStr"/>
-      <c r="U49" t="n">
-        <v>0</v>
-      </c>
-      <c r="V49" t="inlineStr"/>
-      <c r="W49" t="inlineStr">
+      <c r="U49" t="inlineStr"/>
+      <c r="V49" t="n">
+        <v>0</v>
+      </c>
+      <c r="W49" t="inlineStr"/>
+      <c r="X49" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X49" t="inlineStr"/>
+      <c r="Y49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -15469,16 +15447,17 @@
       <c r="P50" t="inlineStr"/>
       <c r="Q50" t="inlineStr"/>
       <c r="R50" t="inlineStr"/>
-      <c r="S50" t="n">
-        <v>1</v>
-      </c>
-      <c r="T50" t="inlineStr"/>
-      <c r="U50" t="n">
-        <v>0</v>
-      </c>
-      <c r="V50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+      <c r="T50" t="n">
+        <v>1</v>
+      </c>
+      <c r="U50" t="inlineStr"/>
+      <c r="V50" t="n">
+        <v>0</v>
+      </c>
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr"/>
+      <c r="Y50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -15533,24 +15512,25 @@
       <c r="N51" t="inlineStr"/>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="n">
+      <c r="Q51" t="inlineStr"/>
+      <c r="R51" t="n">
         <v>2</v>
       </c>
-      <c r="R51" t="inlineStr"/>
-      <c r="S51" t="n">
-        <v>1</v>
-      </c>
-      <c r="T51" t="inlineStr"/>
-      <c r="U51" t="n">
-        <v>0</v>
-      </c>
-      <c r="V51" t="inlineStr"/>
-      <c r="W51" t="inlineStr">
+      <c r="S51" t="inlineStr"/>
+      <c r="T51" t="n">
+        <v>1</v>
+      </c>
+      <c r="U51" t="inlineStr"/>
+      <c r="V51" t="n">
+        <v>0</v>
+      </c>
+      <c r="W51" t="inlineStr"/>
+      <c r="X51" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -15609,16 +15589,17 @@
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="inlineStr"/>
-      <c r="U52" t="n">
-        <v>0</v>
-      </c>
-      <c r="V52" t="inlineStr"/>
-      <c r="W52" t="inlineStr">
+      <c r="U52" t="inlineStr"/>
+      <c r="V52" t="n">
+        <v>0</v>
+      </c>
+      <c r="W52" t="inlineStr"/>
+      <c r="X52" t="inlineStr">
         <is>
           <t>int:2; rangocasteo:5; bonos:2</t>
         </is>
       </c>
-      <c r="X52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -15670,19 +15651,24 @@
         <v>0</v>
       </c>
       <c r="M53" t="inlineStr"/>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Sangrado: Sangrado de 2 HP por turno.</t>
+        </is>
+      </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr"/>
       <c r="Q53" t="inlineStr"/>
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="inlineStr"/>
-      <c r="U53" t="n">
-        <v>0</v>
-      </c>
-      <c r="V53" t="inlineStr"/>
+      <c r="U53" t="inlineStr"/>
+      <c r="V53" t="n">
+        <v>0</v>
+      </c>
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr"/>
+      <c r="Y53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -15734,21 +15720,26 @@
         <v>0</v>
       </c>
       <c r="M54" t="inlineStr"/>
-      <c r="N54" t="n">
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Envenenar: Aplicale Veneno al objetivo.</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
         <v>2</v>
       </c>
-      <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr"/>
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="inlineStr"/>
-      <c r="U54" t="n">
-        <v>0</v>
-      </c>
-      <c r="V54" t="inlineStr"/>
+      <c r="U54" t="inlineStr"/>
+      <c r="V54" t="n">
+        <v>0</v>
+      </c>
       <c r="W54" t="inlineStr"/>
       <c r="X54" t="inlineStr"/>
+      <c r="Y54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -15803,20 +15794,21 @@
       <c r="N55" t="inlineStr"/>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="n">
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="n">
         <v>2</v>
       </c>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="n">
+      <c r="S55" t="inlineStr"/>
+      <c r="T55" t="n">
         <v>3</v>
       </c>
-      <c r="T55" t="inlineStr"/>
-      <c r="U55" t="n">
-        <v>0</v>
-      </c>
-      <c r="V55" t="inlineStr"/>
+      <c r="U55" t="inlineStr"/>
+      <c r="V55" t="n">
+        <v>0</v>
+      </c>
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr"/>
+      <c r="Y55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -15868,21 +15860,26 @@
         <v>0</v>
       </c>
       <c r="M56" t="inlineStr"/>
-      <c r="N56" t="n">
-        <v>1</v>
-      </c>
-      <c r="O56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>Sangrado: Aplicale Sangrado al objetivo.</t>
+        </is>
+      </c>
+      <c r="O56" t="n">
+        <v>1</v>
+      </c>
       <c r="P56" t="inlineStr"/>
       <c r="Q56" t="inlineStr"/>
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="inlineStr"/>
-      <c r="U56" t="n">
-        <v>0</v>
-      </c>
-      <c r="V56" t="inlineStr"/>
+      <c r="U56" t="inlineStr"/>
+      <c r="V56" t="n">
+        <v>0</v>
+      </c>
       <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr"/>
+      <c r="Y56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -15937,20 +15934,21 @@
       <c r="N57" t="inlineStr"/>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="n">
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="n">
         <v>2</v>
       </c>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="n">
+      <c r="S57" t="inlineStr"/>
+      <c r="T57" t="n">
         <v>2</v>
       </c>
-      <c r="T57" t="inlineStr"/>
-      <c r="U57" t="n">
-        <v>0</v>
-      </c>
-      <c r="V57" t="inlineStr"/>
+      <c r="U57" t="inlineStr"/>
+      <c r="V57" t="n">
+        <v>0</v>
+      </c>
       <c r="W57" t="inlineStr"/>
       <c r="X57" t="inlineStr"/>
+      <c r="Y57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -16005,20 +16003,21 @@
       <c r="N58" t="inlineStr"/>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="n">
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="n">
         <v>2</v>
       </c>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="n">
+      <c r="S58" t="inlineStr"/>
+      <c r="T58" t="n">
         <v>3</v>
       </c>
-      <c r="T58" t="inlineStr"/>
-      <c r="U58" t="n">
-        <v>0</v>
-      </c>
-      <c r="V58" t="inlineStr"/>
+      <c r="U58" t="inlineStr"/>
+      <c r="V58" t="n">
+        <v>0</v>
+      </c>
       <c r="W58" t="inlineStr"/>
       <c r="X58" t="inlineStr"/>
+      <c r="Y58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -16070,19 +16069,24 @@
         <v>0</v>
       </c>
       <c r="M59" t="inlineStr"/>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.; Drena vida: Te curás la mitad del daño que hiciste.</t>
+        </is>
+      </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr"/>
       <c r="Q59" t="inlineStr"/>
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="inlineStr"/>
-      <c r="U59" t="n">
-        <v>0</v>
-      </c>
-      <c r="V59" t="inlineStr"/>
+      <c r="U59" t="inlineStr"/>
+      <c r="V59" t="n">
+        <v>0</v>
+      </c>
       <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr"/>
+      <c r="Y59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -16134,19 +16138,24 @@
         <v>0</v>
       </c>
       <c r="M60" t="inlineStr"/>
-      <c r="N60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>Arruina armadura: Aplicale el estado Armadura arruinada al objetivo.</t>
+        </is>
+      </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr"/>
       <c r="Q60" t="inlineStr"/>
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="inlineStr"/>
-      <c r="U60" t="n">
-        <v>0</v>
-      </c>
-      <c r="V60" t="inlineStr"/>
+      <c r="U60" t="inlineStr"/>
+      <c r="V60" t="n">
+        <v>0</v>
+      </c>
       <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr"/>
+      <c r="Y60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -16198,19 +16207,24 @@
         <v>0</v>
       </c>
       <c r="M61" t="inlineStr"/>
-      <c r="N61" t="inlineStr"/>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>Pajaritos: El objetivo queda aturdido (pajaritos).</t>
+        </is>
+      </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr"/>
       <c r="Q61" t="inlineStr"/>
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="inlineStr"/>
-      <c r="U61" t="n">
-        <v>0</v>
-      </c>
-      <c r="V61" t="inlineStr"/>
+      <c r="U61" t="inlineStr"/>
+      <c r="V61" t="n">
+        <v>0</v>
+      </c>
       <c r="W61" t="inlineStr"/>
       <c r="X61" t="inlineStr"/>
+      <c r="Y61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -16262,19 +16276,24 @@
         <v>0</v>
       </c>
       <c r="M62" t="inlineStr"/>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>Envenenar: Veneno de 4 stacks.</t>
+        </is>
+      </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr"/>
       <c r="Q62" t="inlineStr"/>
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="inlineStr"/>
-      <c r="U62" t="n">
-        <v>0</v>
-      </c>
-      <c r="V62" t="inlineStr"/>
+      <c r="U62" t="inlineStr"/>
+      <c r="V62" t="n">
+        <v>0</v>
+      </c>
       <c r="W62" t="inlineStr"/>
       <c r="X62" t="inlineStr"/>
+      <c r="Y62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -16326,19 +16345,24 @@
         <v>0</v>
       </c>
       <c r="M63" t="inlineStr"/>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>Empuje: Lo empuja 2 casilleros (FUE vs CON). Si choca contra algo, daño directo igual a la diferencia.</t>
+        </is>
+      </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr"/>
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="inlineStr"/>
-      <c r="U63" t="n">
-        <v>0</v>
-      </c>
-      <c r="V63" t="inlineStr"/>
+      <c r="U63" t="inlineStr"/>
+      <c r="V63" t="n">
+        <v>0</v>
+      </c>
       <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr"/>
+      <c r="Y63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -16390,25 +16414,30 @@
         <v>0</v>
       </c>
       <c r="M64" t="inlineStr"/>
-      <c r="N64" t="inlineStr"/>
-      <c r="O64" t="n">
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Envenenar: Veneno severo.</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="n">
         <v>2</v>
       </c>
-      <c r="P64" t="inlineStr"/>
       <c r="Q64" t="inlineStr"/>
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="inlineStr"/>
-      <c r="U64" t="n">
-        <v>0</v>
-      </c>
-      <c r="V64" t="inlineStr"/>
-      <c r="W64" t="inlineStr">
+      <c r="U64" t="inlineStr"/>
+      <c r="V64" t="n">
+        <v>0</v>
+      </c>
+      <c r="W64" t="inlineStr"/>
+      <c r="X64" t="inlineStr">
         <is>
           <t>dmg:2</t>
         </is>
       </c>
-      <c r="X64" t="inlineStr"/>
+      <c r="Y64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -16460,19 +16489,24 @@
         <v>0</v>
       </c>
       <c r="M65" t="inlineStr"/>
-      <c r="N65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Ignora armadura 1/2: Si entra, el golpe ignora la Defensa del objetivo.; Drena vida: Te curás tanto HP como el daño que hiciste.</t>
+        </is>
+      </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr"/>
       <c r="Q65" t="inlineStr"/>
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="inlineStr"/>
-      <c r="U65" t="n">
-        <v>0</v>
-      </c>
-      <c r="V65" t="inlineStr"/>
+      <c r="U65" t="inlineStr"/>
+      <c r="V65" t="n">
+        <v>0</v>
+      </c>
       <c r="W65" t="inlineStr"/>
       <c r="X65" t="inlineStr"/>
+      <c r="Y65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -16524,21 +16558,26 @@
         <v>0</v>
       </c>
       <c r="M66" t="inlineStr"/>
-      <c r="N66" t="inlineStr"/>
-      <c r="O66" t="n">
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>Sangrado: Aplicale Sangrado al objetivo.; Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.; Primera sangre: El primer golpe a cada enemigo es doble crítico garantizado.</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr"/>
+      <c r="P66" t="n">
         <v>4</v>
       </c>
-      <c r="P66" t="inlineStr"/>
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="inlineStr"/>
-      <c r="U66" t="n">
-        <v>0</v>
-      </c>
-      <c r="V66" t="inlineStr"/>
+      <c r="U66" t="inlineStr"/>
+      <c r="V66" t="n">
+        <v>0</v>
+      </c>
       <c r="W66" t="inlineStr"/>
       <c r="X66" t="inlineStr"/>
+      <c r="Y66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -16590,19 +16629,24 @@
         <v>0</v>
       </c>
       <c r="M67" t="inlineStr"/>
-      <c r="N67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>Ignora armadura: El golpe ignora la Defensa del objetivo.; Golpes seguidos: Cada golpe seguido al mismo enemigo suma +1 al daño fijo.</t>
+        </is>
+      </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr"/>
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="inlineStr"/>
       <c r="T67" t="inlineStr"/>
-      <c r="U67" t="n">
-        <v>0</v>
-      </c>
-      <c r="V67" t="inlineStr"/>
+      <c r="U67" t="inlineStr"/>
+      <c r="V67" t="n">
+        <v>0</v>
+      </c>
       <c r="W67" t="inlineStr"/>
       <c r="X67" t="inlineStr"/>
+      <c r="Y67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -16654,19 +16698,24 @@
         <v>0</v>
       </c>
       <c r="M68" t="inlineStr"/>
-      <c r="N68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>Arruina armadura: Aplicale el estado Armadura arruinada al objetivo.; Lisiado: Aplicale Lisiado al objetivo.</t>
+        </is>
+      </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr"/>
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="inlineStr"/>
-      <c r="U68" t="n">
-        <v>0</v>
-      </c>
-      <c r="V68" t="inlineStr"/>
+      <c r="U68" t="inlineStr"/>
+      <c r="V68" t="n">
+        <v>0</v>
+      </c>
       <c r="W68" t="inlineStr"/>
       <c r="X68" t="inlineStr"/>
+      <c r="Y68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -16718,19 +16767,24 @@
         <v>0</v>
       </c>
       <c r="M69" t="inlineStr"/>
-      <c r="N69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>Explosión: Daño explosivo en un cono de 3 hex detrás del objetivo.</t>
+        </is>
+      </c>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr"/>
       <c r="Q69" t="inlineStr"/>
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="inlineStr"/>
-      <c r="U69" t="n">
-        <v>0</v>
-      </c>
-      <c r="V69" t="inlineStr"/>
+      <c r="U69" t="inlineStr"/>
+      <c r="V69" t="n">
+        <v>0</v>
+      </c>
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr"/>
+      <c r="Y69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -16782,21 +16836,26 @@
         <v>0</v>
       </c>
       <c r="M70" t="inlineStr"/>
-      <c r="N70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>Media armadura: La mitad del daño ignora la Defensa del objetivo.</t>
+        </is>
+      </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr"/>
       <c r="Q70" t="inlineStr"/>
       <c r="R70" t="inlineStr"/>
-      <c r="S70" t="n">
+      <c r="S70" t="inlineStr"/>
+      <c r="T70" t="n">
         <v>3</v>
       </c>
-      <c r="T70" t="inlineStr"/>
-      <c r="U70" t="n">
-        <v>0</v>
-      </c>
-      <c r="V70" t="inlineStr"/>
+      <c r="U70" t="inlineStr"/>
+      <c r="V70" t="n">
+        <v>0</v>
+      </c>
       <c r="W70" t="inlineStr"/>
       <c r="X70" t="inlineStr"/>
+      <c r="Y70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -16851,20 +16910,21 @@
       <c r="N71" t="inlineStr"/>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="n">
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="n">
         <v>3</v>
       </c>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="n">
+      <c r="S71" t="inlineStr"/>
+      <c r="T71" t="n">
         <v>2</v>
       </c>
-      <c r="T71" t="inlineStr"/>
-      <c r="U71" t="n">
-        <v>0</v>
-      </c>
-      <c r="V71" t="inlineStr"/>
+      <c r="U71" t="inlineStr"/>
+      <c r="V71" t="n">
+        <v>0</v>
+      </c>
       <c r="W71" t="inlineStr"/>
       <c r="X71" t="inlineStr"/>
+      <c r="Y71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -16916,23 +16976,24 @@
         <v>0</v>
       </c>
       <c r="M72" t="inlineStr"/>
-      <c r="N72" t="n">
-        <v>1</v>
-      </c>
-      <c r="O72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
+      <c r="O72" t="n">
+        <v>1</v>
+      </c>
       <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="n">
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="n">
         <v>2</v>
       </c>
-      <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="inlineStr"/>
-      <c r="U72" t="n">
-        <v>0</v>
-      </c>
-      <c r="V72" t="inlineStr"/>
+      <c r="U72" t="inlineStr"/>
+      <c r="V72" t="n">
+        <v>0</v>
+      </c>
       <c r="W72" t="inlineStr"/>
       <c r="X72" t="inlineStr"/>
+      <c r="Y72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -16984,19 +17045,24 @@
         <v>0</v>
       </c>
       <c r="M73" t="inlineStr"/>
-      <c r="N73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr"/>
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="inlineStr"/>
-      <c r="U73" t="n">
-        <v>0</v>
-      </c>
-      <c r="V73" t="inlineStr"/>
+      <c r="U73" t="inlineStr"/>
+      <c r="V73" t="n">
+        <v>0</v>
+      </c>
       <c r="W73" t="inlineStr"/>
       <c r="X73" t="inlineStr"/>
+      <c r="Y73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -17051,20 +17117,21 @@
       <c r="N74" t="inlineStr"/>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr"/>
-      <c r="Q74" t="n">
-        <v>1</v>
-      </c>
-      <c r="R74" t="inlineStr"/>
-      <c r="S74" t="n">
-        <v>1</v>
-      </c>
-      <c r="T74" t="inlineStr"/>
-      <c r="U74" t="n">
-        <v>0</v>
-      </c>
-      <c r="V74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="n">
+        <v>1</v>
+      </c>
+      <c r="S74" t="inlineStr"/>
+      <c r="T74" t="n">
+        <v>1</v>
+      </c>
+      <c r="U74" t="inlineStr"/>
+      <c r="V74" t="n">
+        <v>0</v>
+      </c>
       <c r="W74" t="inlineStr"/>
       <c r="X74" t="inlineStr"/>
+      <c r="Y74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -17116,19 +17183,24 @@
         <v>0</v>
       </c>
       <c r="M75" t="inlineStr"/>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>Ignora 2 de Res. crítico: Al calcular el crítico, el objetivo tiene 2 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr"/>
       <c r="Q75" t="inlineStr"/>
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="inlineStr"/>
-      <c r="U75" t="n">
-        <v>0</v>
-      </c>
-      <c r="V75" t="inlineStr"/>
+      <c r="U75" t="inlineStr"/>
+      <c r="V75" t="n">
+        <v>0</v>
+      </c>
       <c r="W75" t="inlineStr"/>
       <c r="X75" t="inlineStr"/>
+      <c r="Y75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -17180,23 +17252,28 @@
         <v>0</v>
       </c>
       <c r="M76" t="inlineStr"/>
-      <c r="N76" t="inlineStr"/>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr"/>
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="inlineStr"/>
-      <c r="U76" t="n">
-        <v>0</v>
-      </c>
-      <c r="V76" t="inlineStr"/>
-      <c r="W76" t="inlineStr">
+      <c r="U76" t="inlineStr"/>
+      <c r="V76" t="n">
+        <v>0</v>
+      </c>
+      <c r="W76" t="inlineStr"/>
+      <c r="X76" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X76" t="inlineStr"/>
+      <c r="Y76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -17248,23 +17325,24 @@
         <v>0</v>
       </c>
       <c r="M77" t="inlineStr"/>
-      <c r="N77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.; Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr"/>
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="inlineStr"/>
-      <c r="U77" t="n">
-        <v>0</v>
-      </c>
-      <c r="V77" t="inlineStr"/>
+      <c r="U77" t="inlineStr"/>
+      <c r="V77" t="n">
+        <v>0</v>
+      </c>
       <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X77" t="inlineStr"/>
+      <c r="Y77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -17316,19 +17394,24 @@
         <v>0</v>
       </c>
       <c r="M78" t="inlineStr"/>
-      <c r="N78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>Arruina armadura: Aplicale el estado Armadura arruinada al objetivo.</t>
+        </is>
+      </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr"/>
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="inlineStr"/>
-      <c r="U78" t="n">
-        <v>0</v>
-      </c>
-      <c r="V78" t="inlineStr"/>
+      <c r="U78" t="inlineStr"/>
+      <c r="V78" t="n">
+        <v>0</v>
+      </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
+      <c r="Y78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -17380,23 +17463,24 @@
         <v>0</v>
       </c>
       <c r="M79" t="inlineStr"/>
-      <c r="N79" t="n">
+      <c r="N79" t="inlineStr"/>
+      <c r="O79" t="n">
         <v>2</v>
       </c>
-      <c r="O79" t="n">
-        <v>1</v>
-      </c>
-      <c r="P79" t="inlineStr"/>
+      <c r="P79" t="n">
+        <v>1</v>
+      </c>
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="inlineStr"/>
-      <c r="U79" t="n">
-        <v>0</v>
-      </c>
-      <c r="V79" t="inlineStr"/>
+      <c r="U79" t="inlineStr"/>
+      <c r="V79" t="n">
+        <v>0</v>
+      </c>
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr"/>
+      <c r="Y79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -17455,16 +17539,17 @@
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="inlineStr"/>
-      <c r="U80" t="n">
-        <v>0</v>
-      </c>
-      <c r="V80" t="inlineStr"/>
-      <c r="W80" t="inlineStr">
+      <c r="U80" t="inlineStr"/>
+      <c r="V80" t="n">
+        <v>0</v>
+      </c>
+      <c r="W80" t="inlineStr"/>
+      <c r="X80" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X80" t="inlineStr"/>
+      <c r="Y80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -17520,19 +17605,24 @@
           <t>sí</t>
         </is>
       </c>
-      <c r="N81" t="inlineStr"/>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>Prende fuego 1d8: Prende fuego al objetivo: 1d8 por cada stack de fuego.</t>
+        </is>
+      </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr"/>
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="inlineStr"/>
-      <c r="U81" t="n">
-        <v>0</v>
-      </c>
-      <c r="V81" t="inlineStr"/>
+      <c r="U81" t="inlineStr"/>
+      <c r="V81" t="n">
+        <v>0</v>
+      </c>
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr"/>
+      <c r="Y81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -17584,23 +17674,28 @@
         <v>0</v>
       </c>
       <c r="M82" t="inlineStr"/>
-      <c r="N82" t="inlineStr"/>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>Ignora 1 de Res. crítico: Al calcular el crítico, el objetivo tiene 1 menos de resistencia.</t>
+        </is>
+      </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr"/>
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="inlineStr"/>
-      <c r="U82" t="n">
-        <v>0</v>
-      </c>
-      <c r="V82" t="inlineStr"/>
-      <c r="W82" t="inlineStr">
+      <c r="U82" t="inlineStr"/>
+      <c r="V82" t="n">
+        <v>0</v>
+      </c>
+      <c r="W82" t="inlineStr"/>
+      <c r="X82" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X82" t="inlineStr"/>
+      <c r="Y82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -17655,20 +17750,21 @@
       <c r="N83" t="inlineStr"/>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr"/>
-      <c r="Q83" t="n">
+      <c r="Q83" t="inlineStr"/>
+      <c r="R83" t="n">
         <v>2</v>
       </c>
-      <c r="R83" t="inlineStr"/>
-      <c r="S83" t="n">
-        <v>1</v>
-      </c>
-      <c r="T83" t="inlineStr"/>
-      <c r="U83" t="n">
-        <v>0</v>
-      </c>
-      <c r="V83" t="inlineStr"/>
+      <c r="S83" t="inlineStr"/>
+      <c r="T83" t="n">
+        <v>1</v>
+      </c>
+      <c r="U83" t="inlineStr"/>
+      <c r="V83" t="n">
+        <v>0</v>
+      </c>
       <c r="W83" t="inlineStr"/>
       <c r="X83" t="inlineStr"/>
+      <c r="Y83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -17727,20 +17823,17 @@
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr"/>
       <c r="T84" t="inlineStr"/>
-      <c r="U84" t="n">
-        <v>0</v>
-      </c>
-      <c r="V84" t="inlineStr"/>
-      <c r="W84" t="inlineStr">
+      <c r="U84" t="inlineStr"/>
+      <c r="V84" t="n">
+        <v>0</v>
+      </c>
+      <c r="W84" t="inlineStr"/>
+      <c r="X84" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X84" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="Y84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -17799,16 +17892,17 @@
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="inlineStr"/>
-      <c r="U85" t="n">
-        <v>0</v>
-      </c>
-      <c r="V85" t="inlineStr"/>
-      <c r="W85" t="inlineStr">
+      <c r="U85" t="inlineStr"/>
+      <c r="V85" t="n">
+        <v>0</v>
+      </c>
+      <c r="W85" t="inlineStr"/>
+      <c r="X85" t="inlineStr">
         <is>
           <t>rng:1</t>
         </is>
       </c>
-      <c r="X85" t="inlineStr"/>
+      <c r="Y85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -17857,22 +17951,23 @@
       </c>
       <c r="M86" t="inlineStr"/>
       <c r="N86" t="inlineStr"/>
-      <c r="O86" t="n">
+      <c r="O86" t="inlineStr"/>
+      <c r="P86" t="n">
         <v>10</v>
       </c>
-      <c r="P86" t="inlineStr"/>
-      <c r="Q86" t="n">
-        <v>1</v>
-      </c>
-      <c r="R86" t="inlineStr"/>
+      <c r="Q86" t="inlineStr"/>
+      <c r="R86" t="n">
+        <v>1</v>
+      </c>
       <c r="S86" t="inlineStr"/>
       <c r="T86" t="inlineStr"/>
-      <c r="U86" t="n">
-        <v>0</v>
-      </c>
-      <c r="V86" t="inlineStr"/>
+      <c r="U86" t="inlineStr"/>
+      <c r="V86" t="n">
+        <v>0</v>
+      </c>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr"/>
+      <c r="Y86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -17929,16 +18024,17 @@
       <c r="P87" t="inlineStr"/>
       <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr"/>
-      <c r="S87" t="n">
+      <c r="S87" t="inlineStr"/>
+      <c r="T87" t="n">
         <v>3</v>
       </c>
-      <c r="T87" t="inlineStr"/>
-      <c r="U87" t="n">
-        <v>0</v>
-      </c>
-      <c r="V87" t="inlineStr"/>
+      <c r="U87" t="inlineStr"/>
+      <c r="V87" t="n">
+        <v>0</v>
+      </c>
       <c r="W87" t="inlineStr"/>
       <c r="X87" t="inlineStr"/>
+      <c r="Y87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -17990,19 +18086,24 @@
         <v>0</v>
       </c>
       <c r="M88" t="inlineStr"/>
-      <c r="N88" t="inlineStr"/>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" t="inlineStr"/>
       <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="inlineStr"/>
-      <c r="U88" t="n">
-        <v>0</v>
-      </c>
-      <c r="V88" t="inlineStr"/>
+      <c r="U88" t="inlineStr"/>
+      <c r="V88" t="n">
+        <v>0</v>
+      </c>
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr"/>
+      <c r="Y88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -18054,23 +18155,24 @@
         <v>0</v>
       </c>
       <c r="M89" t="inlineStr"/>
-      <c r="N89" t="inlineStr"/>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Rompe armadura 1/2: Aplicale el estado Armadura rota al objetivo.</t>
+        </is>
+      </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr"/>
       <c r="Q89" t="inlineStr"/>
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="inlineStr"/>
       <c r="T89" t="inlineStr"/>
-      <c r="U89" t="n">
-        <v>0</v>
-      </c>
-      <c r="V89" t="inlineStr"/>
+      <c r="U89" t="inlineStr"/>
+      <c r="V89" t="n">
+        <v>0</v>
+      </c>
       <c r="W89" t="inlineStr"/>
-      <c r="X89" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="X89" t="inlineStr"/>
+      <c r="Y89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -18122,22 +18224,27 @@
         <v>0</v>
       </c>
       <c r="M90" t="inlineStr"/>
-      <c r="N90" t="inlineStr"/>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Rompe armadura: Aplicale el estado Armadura rota al objetivo.; Sangrado: Aplicale Sangrado al objetivo.</t>
+        </is>
+      </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr"/>
       <c r="Q90" t="inlineStr"/>
       <c r="R90" t="inlineStr"/>
       <c r="S90" t="inlineStr"/>
       <c r="T90" t="inlineStr"/>
-      <c r="U90" t="n">
-        <v>0</v>
-      </c>
-      <c r="V90" t="inlineStr"/>
+      <c r="U90" t="inlineStr"/>
+      <c r="V90" t="n">
+        <v>0</v>
+      </c>
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr"/>
+      <c r="Y90" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X90"/>
+  <autoFilter ref="A1:Y90"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18535,11 +18642,7 @@
           <t>bloqueo:2</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18603,11 +18706,7 @@
           <t>bloqueo:3</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18671,11 +18770,7 @@
           <t>bloqueo:2</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18737,11 +18832,7 @@
       </c>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18999,11 +19090,7 @@
       </c>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -19675,11 +19762,7 @@
           <t>bloqueo:1</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
+      <c r="V22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -44631,7 +44714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B37"/>
+  <dimension ref="A1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -44759,248 +44842,260 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr"/>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Efectos al golpear</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Lo que el arma hace al pegar, separado por punto y coma. Cada uno: nombre, probabilidad como éxitos/caras (1/2 = 50%, 1/4 = 25%; sin nada = siempre), una tirada extra opcional y, después de dos puntos, qué hace. Ej: Envenenar 1/2: Veneno de 4 stacks; Rompe armadura; Quemadura 1d6</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Columnas de modificadores</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Cada una suma (o resta, con negativo) a ese stat mientras el ítem esté equipado. Vacío = no lo toca.</t>
-        </is>
-      </c>
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>Columnas de modificadores</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Cada una suma (o resta, con negativo) a ese stat mientras el ítem esté equipado. Vacío = no lo toca.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>Otros modificadores</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Para un stat que no tiene columna propia en esa pestaña. Formato: stat:valor; stat:valor — por ejemplo  mov:1; bonos:2</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Consumibles</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Unidades es cuántas trae. Cargas es cuántos usos por unidad. Cura HP suma vida al consumirlo (negativo daña).</t>
-        </is>
-      </c>
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Estado que aplica</t>
+          <t>Consumibles</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Si tiene nombre, al consumir el ítem se activa ese estado alterado. Turnos, HP por turno y Detalle configuran ese estado.</t>
+          <t>Unidades es cuántas trae. Cargas es cuántos usos por unidad. Cura HP suma vida al consumirlo (negativo daña).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Estado que aplica (preset)</t>
+          <t>Estado que aplica</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Opcional, mismo mecanismo que "Estado al equipar (preset)" pero para consumibles. Si el nombre de un preset de la ficha (Afortunado, Coagulación extrema, etc.) va acá, el ítem hereda esa mecánica real al consumirse, aunque "Estado que aplica" tenga otro nombre — así "Coagulación extrema (pergamino)" da inmunidad de verdad en vez de ser solo un cartel.</t>
+          <t>Si tiene nombre, al consumir el ítem se activa ese estado alterado. Turnos, HP por turno y Detalle configuran ese estado.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>Estado que aplica (preset)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Opcional, mismo mecanismo que "Estado al equipar (preset)" pero para consumibles. Si el nombre de un preset de la ficha (Afortunado, Coagulación extrema, etc.) va acá, el ítem hereda esa mecánica real al consumirse, aunque "Estado que aplica" tenga otro nombre — así "Coagulación extrema (pergamino)" da inmunidad de verdad en vez de ser solo un cartel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>Estado permanente</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Con "sí", el estado no vence: queda hasta que el jugador lo borre a mano.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr"/>
-      <c r="B21" s="4" t="inlineStr"/>
-    </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Estado al equipar</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Igual que "Estado que aplica" pero para equipo (armas, escudos, defensivos, accesorios): el estado se activa solo mientras el ítem está puesto y se va al sacárselo — no cuenta turnos.</t>
-        </is>
-      </c>
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>Estado al equipar</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Igual que "Estado que aplica" pero para equipo (armas, escudos, defensivos, accesorios): el estado se activa solo mientras el ítem está puesto y se va al sacárselo — no cuenta turnos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
           <t>Estado al equipar (preset)</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>Opcional. Si el nombre de un preset de la ficha (Afortunado, Sangre pura, etc.) va acá, el ítem hereda esa mecánica real además de mostrar su propio nombre en "Estado al equipar" — así "Afortunado (anillo)" da ventaja de verdad en vez de ser solo un cartel. Dejalo vacío si el efecto no tiene un preset que lo cubra: el estado va a aparecer igual, como recordatorio, pero sin aplicarse solo.</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
-      <c r="B24" s="4" t="inlineStr"/>
-    </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Ocultar del catálogo</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Para ítems generados en automático que todavía no se auditaron ni balancearon: en vez del número, escribí "ocultar en el catálogo" en su celda de Precio (DDE). Ese ítem no se escribe a ficha.html/vendor-generator.html/gm-tools.html — no se puede comprar, no sale en tiendas generadas, no se puede equipar en un creep — pero sigue entero acá y en datos/catalogo.json para irlo revisando. Cuando esté listo, reemplazá el texto por su precio real.</t>
-        </is>
-      </c>
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
+          <t>Ocultar del catálogo</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Para ítems generados en automático que todavía no se auditaron ni balancearon: en vez del número, escribí "ocultar en el catálogo" en su celda de Precio (DDE). Ese ítem no se escribe a ficha.html/vendor-generator.html/gm-tools.html — no se puede comprar, no sale en tiendas generadas, no se puede equipar en un creep — pero sigue entero acá y en datos/catalogo.json para irlo revisando. Cuando esté listo, reemplazá el texto por su precio real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
           <t>Descripción narrativa</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Texto de color: qué se ve, de qué está hecho, su historia. Solo se muestra en la tarjeta que se abre con el botón "Ver". No afecta ninguna mecánica — todo lo que el ítem HACE va en Detalle.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
-    </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="4" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Tiene imagen</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Solo informativo. Las imágenes NO están en este Excel porque pesan cientos de KB cada una; viven en el programa y se conservan solas al reimportar, siempre que no cambies el ID.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr"/>
-    </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>CONTENIDO ACTUAL</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Consumibles</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>146 ítems</t>
-        </is>
-      </c>
+      <c r="B31" s="4" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Armas</t>
+          <t>Consumibles</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>89 ítems</t>
+          <t>146 ítems</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Escudos</t>
+          <t>Armas</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>23 ítems</t>
+          <t>89 ítems</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Defensivos</t>
+          <t>Escudos</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>249 ítems</t>
+          <t>23 ítems</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Accesorios</t>
+          <t>Defensivos</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>72 ítems</t>
+          <t>249 ítems</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
+          <t>Accesorios</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>72 ítems</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>0 ítems</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>579 ítems</t>
         </is>

</xml_diff>

<commit_message>
Catálogo: Pergamino y Poción de Escudo Mágico pasan a Escudo Especial
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/catalogo.xlsx
+++ b/assets/catalogo.xlsx
@@ -7596,7 +7596,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Pergamino de Escudo Mágico</t>
+          <t>Pergamino de Escudo Especial</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Funciona como una barra de HP secundaria de 10 puntos que absorbe daño entrante. Dura todo el combate. Al usarlo se activa el estado 'Escudo mágico (pergamino)'.</t>
+          <t>Funciona como una barra de HP secundaria de 10 puntos que absorbe daño entrante. Dura todo el combate. Al usarlo se activa el estado 'Escudo especial (pergamino)'.</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -7642,7 +7642,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>Escudo mágico (pergamino)</t>
+          <t>Escudo especial (pergamino)</t>
         </is>
       </c>
       <c r="Q98" t="n">
@@ -9506,7 +9506,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Poción de Escudo Mágico</t>
+          <t>Poción de Escudo Especial</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -9530,7 +9530,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Funciona como una barra de HP secundaria de 10 puntos que absorbe daño entrante. Dura 3 turnos. Al consumirla se activa el estado 'Escudo mágico (poción)'.</t>
+          <t>Funciona como una barra de HP secundaria de 10 puntos que absorbe daño entrante. Dura 3 turnos. Al consumirla se activa el estado 'Escudo especial (poción)'.</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -9552,7 +9552,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>Escudo mágico (poción)</t>
+          <t>Escudo especial (poción)</t>
         </is>
       </c>
       <c r="Q123" t="n">

</xml_diff>